<commit_message>
updated message and description in line with CG0184 an closer to rule specification
</commit_message>
<xml_diff>
--- a/rules/CORE-000290/negative/01/data/unit-test-coreid-CG0180-negative.xlsx
+++ b/rules/CORE-000290/negative/01/data/unit-test-coreid-CG0180-negative.xlsx
@@ -1,20 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\els_janssens\CORE\Rule_Authoring\core-contributor\rules\CORE-000290\negative\01\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CA55432-BB02-475E-9B17-7E125ED37D24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Library" sheetId="1" r:id="rId4"/>
-    <sheet name="Datasets" sheetId="2" r:id="rId5"/>
-    <sheet name="Validation" sheetId="3" r:id="rId6"/>
-    <sheet name="lb.xpt" sheetId="4" r:id="rId7"/>
+    <sheet name="Library" sheetId="1" r:id="rId1"/>
+    <sheet name="Datasets" sheetId="2" r:id="rId2"/>
+    <sheet name="Validation" sheetId="3" r:id="rId3"/>
+    <sheet name="lb.xpt" sheetId="4" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="66">
   <si>
     <t>Product</t>
   </si>
@@ -35,9 +44,6 @@
   </si>
   <si>
     <t>lb.xpt</t>
-  </si>
-  <si>
-    <t>Labotory Results</t>
   </si>
   <si>
     <t>Error group</t>
@@ -216,39 +222,29 @@
   </si>
   <si>
     <t>6</t>
+  </si>
+  <si>
+    <t>Laboratory Results</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="0" formatCode="General"/>
-  </numFmts>
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <sz val="15"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b val="1"/>
+      <b/>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <i val="1"/>
+      <i/>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
@@ -455,112 +451,80 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+  </cellStyleXfs>
+  <cellXfs count="30">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-  </cellStyleXfs>
-  <cellXfs count="34">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -570,28 +534,85 @@
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffff0000"/>
-      <rgbColor rgb="ff00ff00"/>
-      <rgbColor rgb="ff0000ff"/>
-      <rgbColor rgb="ffffff00"/>
-      <rgbColor rgb="ffff00ff"/>
-      <rgbColor rgb="ff00ffff"/>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffaaaaaa"/>
-      <rgbColor rgb="ffb2b2b2"/>
-      <rgbColor rgb="ffffffcc"/>
-      <rgbColor rgb="ff9bbb59"/>
-      <rgbColor rgb="fffefb00"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFAAAAAA"/>
+      <rgbColor rgb="FFB2B2B2"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FF9BBB59"/>
+      <rgbColor rgb="FFFEFB00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office Theme">
       <a:dk1>
@@ -717,7 +738,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+            <a:outerShdw blurRad="38100" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -726,7 +747,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+            <a:outerShdw blurRad="38100" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -735,7 +756,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+            <a:outerShdw blurRad="38100" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -809,7 +830,7 @@
           <a:round/>
         </a:ln>
         <a:effectLst>
-          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+          <a:outerShdw blurRad="38100" dist="23000" dir="5400000" rotWithShape="0">
             <a:srgbClr val="000000">
               <a:alpha val="35000"/>
             </a:srgbClr>
@@ -817,7 +838,7 @@
         </a:effectLst>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -835,7 +856,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -864,7 +885,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -889,7 +910,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -914,7 +935,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -939,7 +960,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -964,7 +985,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -989,7 +1010,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1014,7 +1035,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1039,7 +1060,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1064,7 +1085,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1077,9 +1098,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:spDef>
@@ -1094,7 +1121,7 @@
           <a:round/>
         </a:ln>
         <a:effectLst>
-          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+          <a:outerShdw blurRad="38100" dist="23000" dir="5400000" rotWithShape="0">
             <a:srgbClr val="000000">
               <a:alpha val="35000"/>
             </a:srgbClr>
@@ -1102,7 +1129,7 @@
         </a:effectLst>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:noAutofit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1120,7 +1147,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1145,7 +1172,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1170,7 +1197,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1195,7 +1222,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1220,7 +1247,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1245,7 +1272,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1270,7 +1297,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1295,7 +1322,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1320,7 +1347,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1345,7 +1372,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1358,9 +1385,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:lnDef>
@@ -1374,7 +1407,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1392,7 +1425,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1421,7 +1454,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1446,7 +1479,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1471,7 +1504,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1496,7 +1529,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1521,7 +1554,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1546,7 +1579,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1571,7 +1604,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1596,7 +1629,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1621,7 +1654,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1634,106 +1667,51 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:txDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="5" width="8.85156" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.85156" style="1" customWidth="1"/>
+    <col min="1" max="3" width="8.85546875" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.55" customHeight="1">
-      <c r="A1" t="s" s="2">
+    <row r="1" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="2">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-    </row>
-    <row r="2" ht="13.55" customHeight="1">
-      <c r="A2" t="s" s="4">
+    </row>
+    <row r="2" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s" s="4">
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-    </row>
-    <row r="3" ht="13.55" customHeight="1">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-    </row>
-    <row r="4" ht="13.55" customHeight="1">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="5" ht="13.55" customHeight="1">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-    </row>
-    <row r="6" ht="13.55" customHeight="1">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-    </row>
-    <row r="7" ht="13.55" customHeight="1">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-    </row>
-    <row r="8" ht="13.55" customHeight="1">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-    </row>
-    <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-    </row>
-    <row r="10" ht="13.55" customHeight="1">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
@@ -1741,95 +1719,35 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="5" width="8.85156" style="5" customWidth="1"/>
-    <col min="6" max="16384" width="8.85156" style="5" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.55" customHeight="1">
-      <c r="A1" t="s" s="2">
+    <row r="1" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s" s="2">
+      <c r="B1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-    </row>
-    <row r="2" ht="13.55" customHeight="1">
-      <c r="A2" t="s" s="4">
+    </row>
+    <row r="2" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s" s="4">
-        <v>7</v>
-      </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-    </row>
-    <row r="3" ht="13.55" customHeight="1">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-    </row>
-    <row r="4" ht="13.55" customHeight="1">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="5" ht="13.55" customHeight="1">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-    </row>
-    <row r="6" ht="13.55" customHeight="1">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-    </row>
-    <row r="7" ht="13.55" customHeight="1">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-    </row>
-    <row r="8" ht="13.55" customHeight="1">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-    </row>
-    <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-    </row>
-    <row r="10" ht="13.55" customHeight="1">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
+      <c r="B2" s="3" t="s">
+        <v>65</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
@@ -1837,397 +1755,397 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F19"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="6" width="8.85156" style="6" customWidth="1"/>
-    <col min="7" max="16384" width="8.85156" style="6" customWidth="1"/>
+    <col min="1" max="7" width="8.85546875" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.55" customHeight="1">
-      <c r="A1" t="s" s="2">
+    <row r="1" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B1" t="s" s="2">
+      <c r="C1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C1" t="s" s="2">
+      <c r="D1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D1" t="s" s="2">
+      <c r="E1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E1" t="s" s="2">
+      <c r="F1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F1" t="s" s="7">
+    </row>
+    <row r="2" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" ht="13.55" customHeight="1">
-      <c r="A2" s="8">
+      <c r="D2" s="5">
+        <v>5</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5">
         <v>1</v>
       </c>
-      <c r="B2" t="s" s="4">
+      <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s" s="4">
+      <c r="C3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="5">
+        <v>5</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="5">
+        <v>5</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="5">
+        <v>6</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="8">
+      <c r="F5" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="5">
+        <v>6</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
+        <v>2</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="5">
+        <v>6</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="5">
+        <v>7</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5">
+        <v>3</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="5">
+        <v>7</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="5">
+        <v>3</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="5">
+        <v>7</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5">
+        <v>4</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="5">
+        <v>8</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5">
+        <v>4</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="5">
+        <v>8</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5">
+        <v>4</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="5">
+        <v>8</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5">
         <v>5</v>
       </c>
-      <c r="E2" t="s" s="9">
-        <v>15</v>
-      </c>
-      <c r="F2" t="s" s="10">
+      <c r="B14" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="5">
+        <v>9</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5">
+        <v>5</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="5">
+        <v>9</v>
+      </c>
+      <c r="E15" s="8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="3" ht="13.55" customHeight="1">
-      <c r="A3" s="8">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s" s="4">
+      <c r="F15" s="11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="5">
+        <v>5</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" t="s" s="4">
+      <c r="C16" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="5">
+        <v>9</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="5">
+        <v>6</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="5">
+        <v>10</v>
+      </c>
+      <c r="E17" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="8">
-        <v>5</v>
-      </c>
-      <c r="E3" t="s" s="11">
-        <v>17</v>
-      </c>
-      <c r="F3" t="s" s="12">
+      <c r="F17" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="5">
+        <v>6</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="5">
+        <v>10</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="5">
+        <v>6</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="5">
+        <v>10</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" ht="13.55" customHeight="1">
-      <c r="A4" s="8">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D4" s="8">
-        <v>5</v>
-      </c>
-      <c r="E4" t="s" s="9">
-        <v>19</v>
-      </c>
-      <c r="F4" t="s" s="10">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" ht="13.55" customHeight="1">
-      <c r="A5" s="8">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C5" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D5" s="8">
-        <v>6</v>
-      </c>
-      <c r="E5" t="s" s="10">
-        <v>15</v>
-      </c>
-      <c r="F5" t="s" s="13">
+      <c r="F19" s="8" t="s">
         <v>21</v>
-      </c>
-    </row>
-    <row r="6" ht="13.55" customHeight="1">
-      <c r="A6" s="8">
-        <v>2</v>
-      </c>
-      <c r="B6" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C6" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D6" s="8">
-        <v>6</v>
-      </c>
-      <c r="E6" t="s" s="11">
-        <v>17</v>
-      </c>
-      <c r="F6" t="s" s="14">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" ht="13.55" customHeight="1">
-      <c r="A7" s="8">
-        <v>2</v>
-      </c>
-      <c r="B7" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C7" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D7" s="8">
-        <v>6</v>
-      </c>
-      <c r="E7" t="s" s="15">
-        <v>19</v>
-      </c>
-      <c r="F7" t="s" s="12">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" ht="13.55" customHeight="1">
-      <c r="A8" s="8">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C8" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D8" s="8">
-        <v>7</v>
-      </c>
-      <c r="E8" t="s" s="9">
-        <v>15</v>
-      </c>
-      <c r="F8" t="s" s="10">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" s="8">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C9" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D9" s="8">
-        <v>7</v>
-      </c>
-      <c r="E9" t="s" s="11">
-        <v>17</v>
-      </c>
-      <c r="F9" t="s" s="12">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" ht="13.55" customHeight="1">
-      <c r="A10" s="8">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C10" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D10" s="8">
-        <v>7</v>
-      </c>
-      <c r="E10" t="s" s="9">
-        <v>19</v>
-      </c>
-      <c r="F10" t="s" s="10">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" ht="13.55" customHeight="1">
-      <c r="A11" s="8">
-        <v>4</v>
-      </c>
-      <c r="B11" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C11" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D11" s="8">
-        <v>8</v>
-      </c>
-      <c r="E11" t="s" s="10">
-        <v>15</v>
-      </c>
-      <c r="F11" t="s" s="10">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" ht="13.55" customHeight="1">
-      <c r="A12" s="8">
-        <v>4</v>
-      </c>
-      <c r="B12" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C12" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D12" s="8">
-        <v>8</v>
-      </c>
-      <c r="E12" t="s" s="11">
-        <v>17</v>
-      </c>
-      <c r="F12" t="s" s="12">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13" ht="13.55" customHeight="1">
-      <c r="A13" s="8">
-        <v>4</v>
-      </c>
-      <c r="B13" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C13" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D13" s="8">
-        <v>8</v>
-      </c>
-      <c r="E13" t="s" s="15">
-        <v>19</v>
-      </c>
-      <c r="F13" t="s" s="12">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" ht="13.55" customHeight="1">
-      <c r="A14" s="8">
-        <v>5</v>
-      </c>
-      <c r="B14" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C14" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D14" s="8">
-        <v>9</v>
-      </c>
-      <c r="E14" t="s" s="9">
-        <v>15</v>
-      </c>
-      <c r="F14" t="s" s="13">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" ht="13.55" customHeight="1">
-      <c r="A15" s="8">
-        <v>5</v>
-      </c>
-      <c r="B15" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C15" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D15" s="8">
-        <v>9</v>
-      </c>
-      <c r="E15" t="s" s="11">
-        <v>17</v>
-      </c>
-      <c r="F15" t="s" s="14">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" ht="13.55" customHeight="1">
-      <c r="A16" s="8">
-        <v>5</v>
-      </c>
-      <c r="B16" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C16" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D16" s="8">
-        <v>9</v>
-      </c>
-      <c r="E16" t="s" s="9">
-        <v>19</v>
-      </c>
-      <c r="F16" t="s" s="10">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="17" ht="13.55" customHeight="1">
-      <c r="A17" s="8">
-        <v>6</v>
-      </c>
-      <c r="B17" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C17" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D17" s="8">
-        <v>10</v>
-      </c>
-      <c r="E17" t="s" s="10">
-        <v>15</v>
-      </c>
-      <c r="F17" t="s" s="13">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" ht="13.55" customHeight="1">
-      <c r="A18" s="8">
-        <v>6</v>
-      </c>
-      <c r="B18" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C18" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D18" s="8">
-        <v>10</v>
-      </c>
-      <c r="E18" t="s" s="11">
-        <v>17</v>
-      </c>
-      <c r="F18" t="s" s="14">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="19" ht="13.55" customHeight="1">
-      <c r="A19" s="8">
-        <v>6</v>
-      </c>
-      <c r="B19" t="s" s="4">
-        <v>6</v>
-      </c>
-      <c r="C19" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="D19" s="8">
-        <v>10</v>
-      </c>
-      <c r="E19" t="s" s="9">
-        <v>19</v>
-      </c>
-      <c r="F19" t="s" s="11">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
@@ -2235,427 +2153,436 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:M10"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="13" width="8.85156" style="16" customWidth="1"/>
-    <col min="14" max="16384" width="8.85156" style="16" customWidth="1"/>
+    <col min="1" max="4" width="8.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="17.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.42578125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15.28515625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="13.7109375" style="1" customWidth="1"/>
+    <col min="13" max="14" width="8.85546875" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26.55" customHeight="1">
-      <c r="A1" t="s" s="17">
+    <row r="1" spans="1:13" ht="26.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="B1" t="s" s="17">
+      <c r="C1" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="C1" t="s" s="17">
+      <c r="D1" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="D1" t="s" s="17">
+      <c r="E1" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="E1" t="s" s="17">
+      <c r="G1" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="K1" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="L1" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="78.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="H2" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="I2" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="J2" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="K2" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="L2" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="M2" s="14" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="G3" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="H3" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="J3" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="K3" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="L3" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="M3" s="14" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="15">
+        <v>50</v>
+      </c>
+      <c r="B4" s="15">
+        <v>50</v>
+      </c>
+      <c r="C4" s="15">
+        <v>50</v>
+      </c>
+      <c r="D4" s="15">
+        <v>8</v>
+      </c>
+      <c r="E4" s="15">
+        <v>50</v>
+      </c>
+      <c r="F4" s="15">
+        <v>50</v>
+      </c>
+      <c r="G4" s="15">
+        <v>50</v>
+      </c>
+      <c r="H4" s="15">
+        <v>50</v>
+      </c>
+      <c r="I4" s="15">
+        <v>50</v>
+      </c>
+      <c r="J4" s="15">
+        <v>8</v>
+      </c>
+      <c r="K4" s="15">
+        <v>50</v>
+      </c>
+      <c r="L4" s="15">
+        <v>50</v>
+      </c>
+      <c r="M4" s="16">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="17">
+        <v>123101</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="F1" t="s" s="17">
-        <v>31</v>
-      </c>
-      <c r="G1" t="s" s="17">
+      <c r="F5" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="G5" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="H1" t="s" s="17">
-        <v>32</v>
-      </c>
-      <c r="I1" t="s" s="17">
-        <v>33</v>
-      </c>
-      <c r="J1" t="s" s="17">
-        <v>34</v>
-      </c>
-      <c r="K1" t="s" s="17">
-        <v>35</v>
-      </c>
-      <c r="L1" t="s" s="17">
+      <c r="H5" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="L5" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="M1" t="s" s="17">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="2" ht="78.55" customHeight="1">
-      <c r="A2" t="s" s="18">
-        <v>37</v>
-      </c>
-      <c r="B2" t="s" s="18">
-        <v>38</v>
-      </c>
-      <c r="C2" t="s" s="18">
-        <v>39</v>
-      </c>
-      <c r="D2" t="s" s="18">
-        <v>40</v>
-      </c>
-      <c r="E2" t="s" s="18">
-        <v>41</v>
-      </c>
-      <c r="F2" t="s" s="18">
-        <v>42</v>
-      </c>
-      <c r="G2" t="s" s="18">
-        <v>43</v>
-      </c>
-      <c r="H2" t="s" s="18">
-        <v>44</v>
-      </c>
-      <c r="I2" t="s" s="18">
-        <v>45</v>
-      </c>
-      <c r="J2" t="s" s="18">
-        <v>46</v>
-      </c>
-      <c r="K2" t="s" s="18">
-        <v>47</v>
-      </c>
-      <c r="L2" t="s" s="18">
-        <v>48</v>
-      </c>
-      <c r="M2" t="s" s="18">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" ht="13.55" customHeight="1">
-      <c r="A3" t="s" s="18">
-        <v>50</v>
-      </c>
-      <c r="B3" t="s" s="18">
-        <v>50</v>
-      </c>
-      <c r="C3" t="s" s="18">
-        <v>50</v>
-      </c>
-      <c r="D3" t="s" s="18">
+      <c r="M5" s="20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="21">
+        <v>123101</v>
+      </c>
+      <c r="B6" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="E3" t="s" s="18">
-        <v>50</v>
-      </c>
-      <c r="F3" t="s" s="18">
-        <v>50</v>
-      </c>
-      <c r="G3" t="s" s="18">
-        <v>50</v>
-      </c>
-      <c r="H3" t="s" s="18">
-        <v>50</v>
-      </c>
-      <c r="I3" t="s" s="18">
-        <v>50</v>
-      </c>
-      <c r="J3" t="s" s="18">
+      <c r="C6" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="L6" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="M6" s="20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="24">
+        <v>123101</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="K3" t="s" s="18">
-        <v>50</v>
-      </c>
-      <c r="L3" t="s" s="18">
-        <v>50</v>
-      </c>
-      <c r="M3" t="s" s="18">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="4" ht="13.55" customHeight="1">
-      <c r="A4" s="19">
-        <v>50</v>
-      </c>
-      <c r="B4" s="19">
-        <v>50</v>
-      </c>
-      <c r="C4" s="19">
-        <v>50</v>
-      </c>
-      <c r="D4" s="19">
-        <v>8</v>
-      </c>
-      <c r="E4" s="19">
-        <v>50</v>
-      </c>
-      <c r="F4" s="19">
-        <v>50</v>
-      </c>
-      <c r="G4" s="19">
-        <v>50</v>
-      </c>
-      <c r="H4" s="19">
-        <v>50</v>
-      </c>
-      <c r="I4" s="19">
-        <v>50</v>
-      </c>
-      <c r="J4" s="19">
-        <v>8</v>
-      </c>
-      <c r="K4" s="19">
-        <v>50</v>
-      </c>
-      <c r="L4" s="19">
-        <v>50</v>
-      </c>
-      <c r="M4" s="20">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" ht="13.55" customHeight="1">
-      <c r="A5" s="21">
+      <c r="C7" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="G7" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="L7" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="M7" s="20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="17">
         <v>123101</v>
       </c>
-      <c r="B5" t="s" s="11">
+      <c r="B8" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C5" t="s" s="10">
-        <v>53</v>
-      </c>
-      <c r="D5" t="s" s="13">
+      <c r="D8" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="E5" t="s" s="22">
+      <c r="G8" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="K8" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="L8" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="M8" s="20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="27">
+        <v>123101</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="J9" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="K9" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="L9" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="F5" t="s" s="13">
-        <v>55</v>
-      </c>
-      <c r="G5" t="s" s="22">
-        <v>16</v>
-      </c>
-      <c r="H5" t="s" s="13">
-        <v>56</v>
-      </c>
-      <c r="I5" t="s" s="13">
-        <v>57</v>
-      </c>
-      <c r="J5" t="s" s="13">
-        <v>57</v>
-      </c>
-      <c r="K5" t="s" s="13">
-        <v>56</v>
-      </c>
-      <c r="L5" t="s" s="23">
-        <v>18</v>
-      </c>
-      <c r="M5" t="s" s="24">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" ht="39.55" customHeight="1">
-      <c r="A6" s="25">
+      <c r="M9" s="20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="21">
         <v>123101</v>
       </c>
-      <c r="B6" t="s" s="14">
+      <c r="B10" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C6" t="s" s="10">
-        <v>53</v>
-      </c>
-      <c r="D6" t="s" s="9">
+      <c r="D10" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E6" t="s" s="26">
-        <v>22</v>
-      </c>
-      <c r="F6" t="s" s="9">
+      <c r="G10" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="G6" t="s" s="26">
-        <v>21</v>
-      </c>
-      <c r="H6" t="s" s="9">
+      <c r="I10" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="I6" t="s" s="9">
-        <v>61</v>
-      </c>
-      <c r="J6" t="s" s="9">
-        <v>61</v>
-      </c>
-      <c r="K6" t="s" s="9">
+      <c r="J10" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="L6" t="s" s="27">
-        <v>21</v>
-      </c>
-      <c r="M6" t="s" s="24">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" ht="13.55" customHeight="1">
-      <c r="A7" s="28">
-        <v>123101</v>
-      </c>
-      <c r="B7" t="s" s="12">
-        <v>52</v>
-      </c>
-      <c r="C7" t="s" s="10">
-        <v>53</v>
-      </c>
-      <c r="D7" t="s" s="10">
-        <v>62</v>
-      </c>
-      <c r="E7" t="s" s="29">
+      <c r="K10" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="L10" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="F7" t="s" s="10">
-        <v>55</v>
-      </c>
-      <c r="G7" t="s" s="29">
-        <v>23</v>
-      </c>
-      <c r="H7" t="s" s="10">
-        <v>56</v>
-      </c>
-      <c r="I7" t="s" s="10">
-        <v>57</v>
-      </c>
-      <c r="J7" t="s" s="10">
-        <v>57</v>
-      </c>
-      <c r="K7" t="s" s="10">
-        <v>56</v>
-      </c>
-      <c r="L7" t="s" s="30">
-        <v>18</v>
-      </c>
-      <c r="M7" t="s" s="24">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" ht="13.55" customHeight="1">
-      <c r="A8" s="21">
-        <v>123101</v>
-      </c>
-      <c r="B8" t="s" s="11">
-        <v>52</v>
-      </c>
-      <c r="C8" t="s" s="10">
-        <v>53</v>
-      </c>
-      <c r="D8" t="s" s="13">
-        <v>63</v>
-      </c>
-      <c r="E8" t="s" s="22">
+      <c r="M10" s="20" t="s">
         <v>20</v>
-      </c>
-      <c r="F8" t="s" s="13">
-        <v>55</v>
-      </c>
-      <c r="G8" t="s" s="22">
-        <v>24</v>
-      </c>
-      <c r="H8" t="s" s="13">
-        <v>56</v>
-      </c>
-      <c r="I8" t="s" s="13">
-        <v>57</v>
-      </c>
-      <c r="J8" t="s" s="13">
-        <v>57</v>
-      </c>
-      <c r="K8" t="s" s="13">
-        <v>56</v>
-      </c>
-      <c r="L8" t="s" s="23">
-        <v>18</v>
-      </c>
-      <c r="M8" t="s" s="24">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" ht="39.55" customHeight="1">
-      <c r="A9" s="31">
-        <v>123101</v>
-      </c>
-      <c r="B9" t="s" s="4">
-        <v>52</v>
-      </c>
-      <c r="C9" t="s" s="10">
-        <v>53</v>
-      </c>
-      <c r="D9" t="s" s="15">
-        <v>64</v>
-      </c>
-      <c r="E9" t="s" s="32">
-        <v>22</v>
-      </c>
-      <c r="F9" t="s" s="15">
-        <v>59</v>
-      </c>
-      <c r="G9" t="s" s="32">
-        <v>25</v>
-      </c>
-      <c r="H9" t="s" s="15">
-        <v>60</v>
-      </c>
-      <c r="I9" t="s" s="15">
-        <v>61</v>
-      </c>
-      <c r="J9" t="s" s="15">
-        <v>61</v>
-      </c>
-      <c r="K9" t="s" s="15">
-        <v>60</v>
-      </c>
-      <c r="L9" t="s" s="33">
-        <v>21</v>
-      </c>
-      <c r="M9" t="s" s="24">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" ht="39.55" customHeight="1">
-      <c r="A10" s="25">
-        <v>123101</v>
-      </c>
-      <c r="B10" t="s" s="14">
-        <v>52</v>
-      </c>
-      <c r="C10" t="s" s="10">
-        <v>53</v>
-      </c>
-      <c r="D10" t="s" s="9">
-        <v>65</v>
-      </c>
-      <c r="E10" t="s" s="26">
-        <v>22</v>
-      </c>
-      <c r="F10" t="s" s="9">
-        <v>59</v>
-      </c>
-      <c r="G10" t="s" s="26">
-        <v>26</v>
-      </c>
-      <c r="H10" t="s" s="9">
-        <v>60</v>
-      </c>
-      <c r="I10" t="s" s="9">
-        <v>61</v>
-      </c>
-      <c r="J10" t="s" s="9">
-        <v>61</v>
-      </c>
-      <c r="K10" t="s" s="9">
-        <v>60</v>
-      </c>
-      <c r="L10" t="s" s="27">
-        <v>21</v>
-      </c>
-      <c r="M10" t="s" s="24">
-        <v>21</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>